<commit_message>
Add PDF export of the capacity model and A4 print layout
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017gaAdEpfwPoXxk1QkReCcV
</commit_message>
<xml_diff>
--- a/model/Veolia_capacity_2027.xlsx
+++ b/model/Veolia_capacity_2027.xlsx
@@ -17,6 +17,9 @@
     <sheet name="Tornado" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Rating" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Area" vbProcedure="false">Engine!$A$1:$E$70</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -1825,7 +1828,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1938,7 +1941,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1949,7 +1952,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2318,7 +2321,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2329,7 +2332,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3766,7 +3769,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3777,7 +3780,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4199,7 +4202,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4210,7 +4213,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4494,7 +4497,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4505,7 +4508,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AA70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -11642,7 +11645,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -11653,7 +11656,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -12238,7 +12241,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -12249,7 +12252,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -12335,7 +12338,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>